<commit_message>
add new employee status
</commit_message>
<xml_diff>
--- a/For Google Sheets - AiEmployeeTest.xlsx
+++ b/For Google Sheets - AiEmployeeTest.xlsx
@@ -839,7 +839,16 @@
       <c r="M5" s="20" t="n"/>
       <c r="N5" s="20" t="n"/>
       <c r="O5" s="20" t="n"/>
-      <c r="Q5" s="3" t="n"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Статус «Не участвует»:</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>сотрудник остаётся в таблице со своей историей, но в волне не участвует: войти не может, при startNewWave не сбрасывается, в статистику не попадает. Строку не удалять — на ID завязаны Results, Employees_history и Usages.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n"/>
@@ -18665,7 +18674,7 @@
   <autoFilter ref="A1:Y995"/>
   <dataValidations count="2">
     <dataValidation sqref="F2:F995" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Использован,Не использован,Частично"</formula1>
+      <formula1>"Использован,Не использован,Частично,Не участвует"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N995" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Энтузиаст,Конформист,Оппонент"</formula1>

</xml_diff>